<commit_message>
Corrections in main dofile, updates in public revenue and tobacco consumption with ECV
</commit_message>
<xml_diff>
--- a/Indicators/Alcohol.xlsx
+++ b/Indicators/Alcohol.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uredu.sharepoint.com/sites/ControlTabacoFacultadEconomica/Documentos compartidos/Monitoreo/ALCOHOL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uredu.sharepoint.com/sites/ControlTabacoFacultadEconomica/Documentos compartidos/Monitoreo/Repositorio/Indicators/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="740" documentId="8_{D2B865D6-6803-4024-9496-7B13481E7340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41DD5E5E-857D-4AC6-A7EC-4416E68A64F8}"/>
+  <xr:revisionPtr revIDLastSave="742" documentId="8_{D2B865D6-6803-4024-9496-7B13481E7340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AF11CD8-68A7-475B-BF1B-4D7EBD320552}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{7A94D5C5-EB71-44F3-BD13-919ACF62FAE6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{7A94D5C5-EB71-44F3-BD13-919ACF62FAE6}"/>
   </bookViews>
   <sheets>
     <sheet name="Salud" sheetId="6" r:id="rId1"/>
@@ -1600,14 +1600,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="8">
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="###,###.00"/>
-    <numFmt numFmtId="166" formatCode="##,#00"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
-    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="###,###.00"/>
+    <numFmt numFmtId="165" formatCode="##,#00"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
   <fonts count="21" x14ac:knownFonts="1">
     <font>
@@ -1903,7 +1903,7 @@
   <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
@@ -1914,7 +1914,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1925,34 +1925,34 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="4" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="7">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="7">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1967,7 +1967,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="11" fillId="6" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1989,25 +1989,25 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8"/>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="13" fillId="11" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="13" fillId="11" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="9" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2017,10 +2017,10 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -6603,7 +6603,7 @@
             <c:numRef>
               <c:f>'Precio alcohol (destilados)'!$S$2:$S$10</c:f>
               <c:numCache>
-                <c:formatCode>_-"$"\ * #,##0.00_-;\-"$"\ * #,##0.00_-;_-"$"\ * "-"??_-;_-@_-</c:formatCode>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>14.169347412061448</c:v>
@@ -6885,7 +6885,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-" sourceLinked="1"/>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -7094,7 +7094,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="es-MX"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -7473,7 +7473,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="es-MX"/>
+              <a:endParaRPr lang="es-419"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -7575,7 +7575,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="es-MX"/>
+              <a:endParaRPr lang="es-419"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -12810,7 +12810,7 @@
             <c:numRef>
               <c:f>'Precio alcohol (cerveza)'!$U$3:$U$10</c:f>
               <c:numCache>
-                <c:formatCode>_-"$"\ * #,##0.00_-;\-"$"\ * #,##0.00_-;_-"$"\ * "-"??_-;_-@_-</c:formatCode>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>1.8390106547582652</c:v>
@@ -13089,7 +13089,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-" sourceLinked="1"/>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -13657,7 +13657,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="es-MX"/>
+              <a:endParaRPr lang="es-419"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -13759,7 +13759,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="es-MX"/>
+              <a:endParaRPr lang="es-419"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -14737,7 +14737,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="es-MX"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -22965,89 +22965,6 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Tamaño Mercado Alcohol'!#REF!</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>#REF!</c:v>
-                </c:pt>
-              </c:strCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Tamaño Mercado Alcohol'!$A$2:$A$10</c:f>
-              <c:strCache>
-                <c:ptCount val="9"/>
-                <c:pt idx="0">
-                  <c:v>2014</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2015</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2016</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2017</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2018</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2019</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2020</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>2021</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>2022</c:v>
-                </c:pt>
-              </c:strCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Tamaño Mercado Alcohol'!#REF!</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D821-4BDB-8525-4A76421E0745}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
           <c:idx val="5"/>
           <c:order val="5"/>
           <c:tx>
@@ -23273,21 +23190,21 @@
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
             <c15:filteredLineSeries>
               <c15:ser>
-                <c:idx val="1"/>
-                <c:order val="1"/>
+                <c:idx val="0"/>
+                <c:order val="0"/>
                 <c:tx>
                   <c:strRef>
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>'Tamaño Mercado Alcohol'!$B$1</c15:sqref>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!#REF!</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:strCache>
                       <c:ptCount val="1"/>
                       <c:pt idx="0">
-                        <c:v>Tamaño mercado Euromonitor</c:v>
+                        <c:v>#REF!</c:v>
                       </c:pt>
                     </c:strCache>
                   </c:strRef>
@@ -23295,7 +23212,7 @@
                 <c:spPr>
                   <a:ln w="28575" cap="rnd">
                     <a:solidFill>
-                      <a:schemeClr val="accent2"/>
+                      <a:schemeClr val="accent1"/>
                     </a:solidFill>
                     <a:round/>
                   </a:ln>
@@ -23350,6 +23267,106 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!#REF!</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>1</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-D821-4BDB-8525-4A76421E0745}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredLineSeries>
+            <c15:filteredLineSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!$B$1</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>Tamaño mercado Euromonitor</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent2"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!$A$2:$A$10</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="9"/>
+                      <c:pt idx="0">
+                        <c:v>2014</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>2015</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>2016</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>2017</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>2018</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>2019</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>2020</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>2021</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>2022</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
                           <c15:sqref>'Tamaño Mercado Alcohol'!$B$2:$B$10</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
@@ -23388,7 +23405,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000000-1B92-459E-975A-BFB996CF650F}"/>
                   </c:ext>
@@ -23893,7 +23910,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -24031,178 +24048,6 @@
       <c:lineChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Tamaño Mercado Alcohol'!#REF!</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>#REF!</c:v>
-                </c:pt>
-              </c:strCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Tamaño Mercado Alcohol'!$A$2:$A$11</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>2014</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2015</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2016</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2017</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2018</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2019</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2020</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>2021</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2023</c:v>
-                </c:pt>
-              </c:strCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Tamaño Mercado Alcohol'!#REF!</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-1FA6-4F2F-9D51-BB55474D3C69}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Tamaño Mercado Alcohol'!#REF!</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>#REF!</c:v>
-                </c:pt>
-              </c:strCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Tamaño Mercado Alcohol'!$A$2:$A$11</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>2014</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2015</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2016</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2017</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2018</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2019</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2020</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>2021</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>2022</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2023</c:v>
-                </c:pt>
-              </c:strCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Tamaño Mercado Alcohol'!#REF!</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-1FA6-4F2F-9D51-BB55474D3C69}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
         <c:ser>
           <c:idx val="9"/>
           <c:order val="9"/>
@@ -24448,6 +24293,212 @@
                 <c:extLst>
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000000-1FA6-4F2F-9D51-BB55474D3C69}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredLineSeries>
+            <c15:filteredLineSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!#REF!</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>#REF!</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent2"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!$A$2:$A$11</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="10"/>
+                      <c:pt idx="0">
+                        <c:v>2014</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>2015</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>2016</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>2017</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>2018</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>2019</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>2020</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>2021</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>2022</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>2023</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!#REF!</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>1</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-1FA6-4F2F-9D51-BB55474D3C69}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredLineSeries>
+            <c15:filteredLineSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!#REF!</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>#REF!</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!$A$2:$A$11</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="10"/>
+                      <c:pt idx="0">
+                        <c:v>2014</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>2015</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>2016</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>2017</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>2018</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>2019</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>2020</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>2021</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>2022</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>2023</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Tamaño Mercado Alcohol'!#REF!</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>1</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-1FA6-4F2F-9D51-BB55474D3C69}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -25347,7 +25398,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -25546,7 +25597,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="es-MX"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -27708,7 +27759,7 @@
             <c:numRef>
               <c:f>'Precio alcohol (vino)'!$S$2:$S$10</c:f>
               <c:numCache>
-                <c:formatCode>_-"$"\ * #,##0.00_-;\-"$"\ * #,##0.00_-;_-"$"\ * "-"??_-;_-@_-</c:formatCode>
+                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>6.9276134081626077</c:v>
@@ -27928,7 +27979,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="r"/>
-        <c:numFmt formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-" sourceLinked="1"/>
+        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -28523,7 +28574,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="es-MX"/>
+              <a:endParaRPr lang="es-419"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -28626,7 +28677,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="es-MX"/>
+              <a:endParaRPr lang="es-419"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -43996,16 +44047,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9EBD662-458C-4DF7-9B69-EFEE5705659C}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.85546875" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="86.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="86.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -44028,7 +44079,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2014</v>
       </c>
@@ -44051,7 +44102,7 @@
         <v>0.19571987000955501</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2015</v>
       </c>
@@ -44074,7 +44125,7 @@
         <v>0.197631075162399</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2016</v>
       </c>
@@ -44097,7 +44148,7 @@
         <v>0.195417392839423</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2017</v>
       </c>
@@ -44120,7 +44171,7 @@
         <v>0.19965602618450301</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2018</v>
       </c>
@@ -44143,7 +44194,7 @@
         <v>0.19908742762841899</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2019</v>
       </c>
@@ -44166,7 +44217,7 @@
         <v>0.14550250789357799</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2020</v>
       </c>
@@ -44186,7 +44237,7 @@
         <v>0.19929015896014601</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -44206,12 +44257,12 @@
         <v>0.16740480817509401</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2022</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2023</v>
       </c>
@@ -44225,19 +44276,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0434DCFB-BB37-495B-AE13-9B3B42412A64}">
   <dimension ref="A1:O21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" customWidth="1"/>
-    <col min="9" max="9" width="16.42578125" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" customWidth="1"/>
+    <col min="7" max="7" width="19.44140625" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" customWidth="1"/>
+    <col min="9" max="9" width="16.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -44269,7 +44320,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -44299,7 +44350,7 @@
         <v>82.47</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -44329,7 +44380,7 @@
         <v>88.05</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -44362,7 +44413,7 @@
         <v>93.11</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -44395,7 +44446,7 @@
         <v>96.92</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -44428,7 +44479,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -44461,7 +44512,7 @@
         <v>103.8</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
@@ -44494,7 +44545,7 @@
         <v>105.48</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -44527,7 +44578,7 @@
         <v>111.41</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
@@ -44557,7 +44608,7 @@
         <v>126.03</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
@@ -44575,7 +44626,7 @@
         <v>137.72</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C13" s="60"/>
       <c r="D13" s="60"/>
       <c r="L13" s="61"/>
@@ -44583,35 +44634,35 @@
       <c r="N13" s="61"/>
       <c r="O13" s="61"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="27"/>
       <c r="B14" s="27"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="27"/>
       <c r="B15" s="27"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="27"/>
       <c r="B16" s="27"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="27"/>
       <c r="B17" s="27"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="27"/>
       <c r="B18" s="27"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="27"/>
       <c r="B19" s="27"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="27"/>
       <c r="B20" s="27"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="27"/>
       <c r="B21" s="27"/>
     </row>
@@ -44628,24 +44679,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD10DE07-3460-400A-8F12-19CC5985E2D3}">
   <dimension ref="A1:Z17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" customWidth="1"/>
-    <col min="7" max="15" width="9.140625"/>
-    <col min="16" max="16" width="14.7109375" customWidth="1"/>
-    <col min="17" max="17" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.140625"/>
-    <col min="19" max="19" width="11.85546875" customWidth="1"/>
-    <col min="20" max="20" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.140625"/>
-    <col min="23" max="25" width="13.85546875" customWidth="1"/>
-    <col min="26" max="28" width="13.7109375" customWidth="1"/>
+    <col min="2" max="4" width="15.6640625" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" customWidth="1"/>
+    <col min="7" max="15" width="9.109375"/>
+    <col min="16" max="16" width="14.6640625" customWidth="1"/>
+    <col min="17" max="17" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.109375"/>
+    <col min="19" max="19" width="11.88671875" customWidth="1"/>
+    <col min="20" max="20" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.109375"/>
+    <col min="23" max="25" width="13.88671875" customWidth="1"/>
+    <col min="26" max="28" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="105" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -44717,7 +44768,7 @@
       </c>
       <c r="X1" s="7"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -44803,7 +44854,7 @@
       </c>
       <c r="X2" s="9"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2016</v>
       </c>
@@ -44888,7 +44939,7 @@
       </c>
       <c r="X3" s="9"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2017</v>
       </c>
@@ -44976,7 +45027,7 @@
       </c>
       <c r="X4" s="9"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -45064,7 +45115,7 @@
       </c>
       <c r="X5" s="9"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2019</v>
       </c>
@@ -45152,7 +45203,7 @@
       </c>
       <c r="X6" s="9"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2020</v>
       </c>
@@ -45240,7 +45291,7 @@
       </c>
       <c r="X7" s="9"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -45328,7 +45379,7 @@
       </c>
       <c r="X8" s="9"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -45416,7 +45467,7 @@
       </c>
       <c r="X9" s="9"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2023</v>
       </c>
@@ -45500,19 +45551,19 @@
       </c>
       <c r="X10" s="9"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="H11" s="4">
         <f>E11-E11/1.19</f>
         <v>0</v>
       </c>
       <c r="V11" s="6"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C14" s="40" t="s">
         <v>46</v>
       </c>
@@ -45530,7 +45581,7 @@
       <c r="W14" s="14"/>
       <c r="Y14" s="6"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="S15" s="22" t="s">
         <v>48</v>
       </c>
@@ -45544,10 +45595,10 @@
         <v>-1.5390419094370058E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="S16" s="19"/>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>49</v>
       </c>
@@ -45569,21 +45620,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{133254FF-F683-484E-B56C-1EED7F2EDCBF}">
   <dimension ref="A1:Z16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="4" width="17.28515625" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" customWidth="1"/>
-    <col min="17" max="17" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.85546875" customWidth="1"/>
-    <col min="20" max="20" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="25" width="13.85546875" customWidth="1"/>
-    <col min="26" max="28" width="13.7109375" customWidth="1"/>
+    <col min="3" max="4" width="17.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" customWidth="1"/>
+    <col min="16" max="16" width="14.6640625" customWidth="1"/>
+    <col min="17" max="17" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.88671875" customWidth="1"/>
+    <col min="20" max="20" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="25" width="13.88671875" customWidth="1"/>
+    <col min="26" max="28" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="72" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -45655,7 +45706,7 @@
       </c>
       <c r="X1" s="7"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -45738,7 +45789,7 @@
       </c>
       <c r="X2" s="9"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2016</v>
       </c>
@@ -45820,7 +45871,7 @@
       </c>
       <c r="X3" s="9"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2017</v>
       </c>
@@ -45908,7 +45959,7 @@
       </c>
       <c r="X4" s="9"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -45996,7 +46047,7 @@
       </c>
       <c r="X5" s="9"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2019</v>
       </c>
@@ -46084,7 +46135,7 @@
       </c>
       <c r="X6" s="9"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2020</v>
       </c>
@@ -46172,7 +46223,7 @@
       </c>
       <c r="X7" s="9"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -46260,7 +46311,7 @@
       </c>
       <c r="X8" s="9"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -46348,7 +46399,7 @@
       </c>
       <c r="X9" s="9"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2023</v>
       </c>
@@ -46432,19 +46483,19 @@
       </c>
       <c r="X10" s="9"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="H11" s="4">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="W11" s="6"/>
     </row>
-    <row r="13" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="C14" s="40" t="s">
         <v>46</v>
       </c>
@@ -46462,7 +46513,7 @@
       <c r="W14" s="14"/>
       <c r="Y14" s="6"/>
     </row>
-    <row r="15" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S15" s="22" t="s">
         <v>48</v>
       </c>
@@ -46476,7 +46527,7 @@
         <v>-0.27047798142535417</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="H16">
         <f>H10/J10</f>
         <v>0.70551676182906686</v>
@@ -46500,15 +46551,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61A8C809-19CC-4C44-A17E-2B5A22492F50}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="16.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="16.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="94.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -46534,7 +46585,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2014</v>
       </c>
@@ -46551,7 +46602,7 @@
         <v>1.02</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2015</v>
       </c>
@@ -46568,7 +46619,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2016</v>
       </c>
@@ -46588,7 +46639,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2017</v>
       </c>
@@ -46608,7 +46659,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2018</v>
       </c>
@@ -46625,7 +46676,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2019</v>
       </c>
@@ -46649,7 +46700,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2020</v>
       </c>
@@ -46673,7 +46724,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2021</v>
       </c>
@@ -46697,7 +46748,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2022</v>
       </c>
@@ -46715,7 +46766,7 @@
         <v>682.12689</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2023</v>
       </c>
@@ -46739,22 +46790,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDBBAC2C-0EF5-46F8-8124-675BFA7921E7}">
   <dimension ref="A1:AA16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="6" width="14.28515625" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" customWidth="1"/>
-    <col min="17" max="17" width="14.7109375" customWidth="1"/>
-    <col min="18" max="18" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.85546875" customWidth="1"/>
-    <col min="21" max="21" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="26" width="13.85546875" customWidth="1"/>
-    <col min="27" max="29" width="13.7109375" customWidth="1"/>
+    <col min="3" max="4" width="15.6640625" customWidth="1"/>
+    <col min="5" max="6" width="14.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.5546875" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" customWidth="1"/>
+    <col min="17" max="17" width="14.6640625" customWidth="1"/>
+    <col min="18" max="18" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.88671875" customWidth="1"/>
+    <col min="21" max="21" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="26" width="13.88671875" customWidth="1"/>
+    <col min="27" max="29" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="72" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -46832,7 +46883,7 @@
       </c>
       <c r="Z1" s="45"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -46903,7 +46954,7 @@
       <c r="Y2" s="54"/>
       <c r="Z2" s="46"/>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2016</v>
       </c>
@@ -46994,7 +47045,7 @@
       </c>
       <c r="Z3" s="46"/>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2017</v>
       </c>
@@ -47085,7 +47136,7 @@
       </c>
       <c r="Z4" s="46"/>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -47176,7 +47227,7 @@
       </c>
       <c r="Z5" s="46"/>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2019</v>
       </c>
@@ -47267,7 +47318,7 @@
       </c>
       <c r="Z6" s="46"/>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2020</v>
       </c>
@@ -47358,7 +47409,7 @@
       </c>
       <c r="Z7" s="46"/>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -47449,7 +47500,7 @@
       </c>
       <c r="Z8" s="46"/>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -47540,7 +47591,7 @@
       </c>
       <c r="Z9" s="46"/>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2023</v>
       </c>
@@ -47626,15 +47677,15 @@
       </c>
       <c r="Z10" s="46"/>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="X11" s="6"/>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C14" s="40" t="s">
         <v>46</v>
       </c>
@@ -47652,7 +47703,7 @@
       <c r="X14" s="14"/>
       <c r="Z14" s="6"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="T15" s="22" t="s">
         <v>48</v>
       </c>
@@ -47666,7 +47717,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C16" s="44" t="s">
         <v>80</v>
       </c>
@@ -47696,17 +47747,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0E166C0-BC0E-4B17-B07D-A8B34EF05B11}">
   <dimension ref="A1:J289"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="9.140625" style="37" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" style="37" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="37" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="37" customWidth="1"/>
-    <col min="7" max="256" width="9.140625" style="37" customWidth="1"/>
-    <col min="257" max="16384" width="11.42578125" style="37"/>
+    <col min="1" max="3" width="9.109375" style="37" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" style="37" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="37" customWidth="1"/>
+    <col min="6" max="6" width="17.33203125" style="37" customWidth="1"/>
+    <col min="7" max="256" width="9.109375" style="37" customWidth="1"/>
+    <col min="257" max="16384" width="11.44140625" style="37"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
         <v>22</v>
       </c>
@@ -47726,7 +47777,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="37" t="s">
         <v>86</v>
       </c>
@@ -47746,7 +47797,7 @@
         <v>30.330000000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="37" t="s">
         <v>86</v>
       </c>
@@ -47766,7 +47817,7 @@
         <v>30.889999999999993</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="37" t="s">
         <v>86</v>
       </c>
@@ -47786,7 +47837,7 @@
         <v>31.33</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="s">
         <v>86</v>
       </c>
@@ -47806,7 +47857,7 @@
         <v>31.499999999999993</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
         <v>86</v>
       </c>
@@ -47826,7 +47877,7 @@
         <v>31.379999999999995</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
         <v>86</v>
       </c>
@@ -47846,7 +47897,7 @@
         <v>31.289999999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
         <v>86</v>
       </c>
@@ -47866,7 +47917,7 @@
         <v>31.47</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
         <v>86</v>
       </c>
@@ -47886,7 +47937,7 @@
         <v>31.789999999999996</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
         <v>86</v>
       </c>
@@ -47906,7 +47957,7 @@
         <v>32.36</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
         <v>86</v>
       </c>
@@ -47926,7 +47977,7 @@
         <v>32.639999999999993</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
         <v>86</v>
       </c>
@@ -47946,7 +47997,7 @@
         <v>32.61999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="37" t="s">
         <v>86</v>
       </c>
@@ -47966,7 +48017,7 @@
         <v>32.700000000000003</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="37" t="s">
         <v>111</v>
       </c>
@@ -47986,7 +48037,7 @@
         <v>33.279999999999994</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
         <v>111</v>
       </c>
@@ -48006,7 +48057,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
         <v>111</v>
       </c>
@@ -48026,7 +48077,7 @@
         <v>34.559999999999995</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
         <v>111</v>
       </c>
@@ -48046,7 +48097,7 @@
         <v>34.909999999999997</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="37" t="s">
         <v>111</v>
       </c>
@@ -48066,7 +48117,7 @@
         <v>35.159999999999989</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="37" t="s">
         <v>111</v>
       </c>
@@ -48086,7 +48137,7 @@
         <v>35.380000000000003</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="37" t="s">
         <v>111</v>
       </c>
@@ -48106,7 +48157,7 @@
         <v>35.459999999999994</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="37" t="s">
         <v>111</v>
       </c>
@@ -48126,7 +48177,7 @@
         <v>35.520000000000003</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="37" t="s">
         <v>111</v>
       </c>
@@ -48146,7 +48197,7 @@
         <v>35.559999999999995</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="37" t="s">
         <v>111</v>
       </c>
@@ -48166,7 +48217,7 @@
         <v>35.529999999999994</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="37" t="s">
         <v>111</v>
       </c>
@@ -48191,7 +48242,7 @@
       <c r="I24" s="39"/>
       <c r="J24" s="39"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="37" t="s">
         <v>111</v>
       </c>
@@ -48211,7 +48262,7 @@
         <v>35.669999999999995</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="37" t="s">
         <v>125</v>
       </c>
@@ -48231,7 +48282,7 @@
         <v>35.709999999999994</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="37" t="s">
         <v>125</v>
       </c>
@@ -48251,7 +48302,7 @@
         <v>35.919999999999995</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="37" t="s">
         <v>125</v>
       </c>
@@ -48271,7 +48322,7 @@
         <v>35.99</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="37" t="s">
         <v>125</v>
       </c>
@@ -48291,7 +48342,7 @@
         <v>36.069999999999993</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="37" t="s">
         <v>125</v>
       </c>
@@ -48311,7 +48362,7 @@
         <v>36.319999999999993</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="37" t="s">
         <v>125</v>
       </c>
@@ -48331,7 +48382,7 @@
         <v>36.929999999999993</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="37" t="s">
         <v>125</v>
       </c>
@@ -48351,7 +48402,7 @@
         <v>37.64</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="37" t="s">
         <v>125</v>
       </c>
@@ -48371,7 +48422,7 @@
         <v>38.159999999999997</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="37" t="s">
         <v>125</v>
       </c>
@@ -48391,7 +48442,7 @@
         <v>38.6</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="37" t="s">
         <v>125</v>
       </c>
@@ -48411,7 +48462,7 @@
         <v>38.78</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="37" t="s">
         <v>125</v>
       </c>
@@ -48431,7 +48482,7 @@
         <v>38.839999999999996</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="37" t="s">
         <v>125</v>
       </c>
@@ -48451,7 +48502,7 @@
         <v>38.849999999999994</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="37" t="s">
         <v>138</v>
       </c>
@@ -48471,7 +48522,7 @@
         <v>39.089999999999996</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="37" t="s">
         <v>138</v>
       </c>
@@ -48491,7 +48542,7 @@
         <v>39.78</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="37" t="s">
         <v>138</v>
       </c>
@@ -48511,7 +48562,7 @@
         <v>40.319999999999993</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="37" t="s">
         <v>138</v>
       </c>
@@ -48531,7 +48582,7 @@
         <v>40.449999999999996</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="37" t="s">
         <v>138</v>
       </c>
@@ -48551,7 +48602,7 @@
         <v>40.54999999999999</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="37" t="s">
         <v>138</v>
       </c>
@@ -48571,7 +48622,7 @@
         <v>40.619999999999997</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="37" t="s">
         <v>138</v>
       </c>
@@ -48591,7 +48642,7 @@
         <v>40.659999999999989</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="37" t="s">
         <v>138</v>
       </c>
@@ -48611,7 +48662,7 @@
         <v>40.879999999999995</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="37" t="s">
         <v>138</v>
       </c>
@@ -48631,7 +48682,7 @@
         <v>41.15</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="37" t="s">
         <v>138</v>
       </c>
@@ -48651,7 +48702,7 @@
         <v>41.3</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="37" t="s">
         <v>138</v>
       </c>
@@ -48671,7 +48722,7 @@
         <v>41.49</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="37" t="s">
         <v>138</v>
       </c>
@@ -48691,7 +48742,7 @@
         <v>41.599999999999994</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="37" t="s">
         <v>151</v>
       </c>
@@ -48711,7 +48762,7 @@
         <v>41.939999999999991</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="37" t="s">
         <v>151</v>
       </c>
@@ -48731,7 +48782,7 @@
         <v>42.539999999999992</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="37" t="s">
         <v>151</v>
       </c>
@@ -48751,7 +48802,7 @@
         <v>43.13</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="37" t="s">
         <v>151</v>
       </c>
@@ -48771,7 +48822,7 @@
         <v>43.349999999999994</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="37" t="s">
         <v>151</v>
       </c>
@@ -48791,7 +48842,7 @@
         <v>43.429999999999993</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="37" t="s">
         <v>151</v>
       </c>
@@ -48811,7 +48862,7 @@
         <v>43.55</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="37" t="s">
         <v>151</v>
       </c>
@@ -48831,7 +48882,7 @@
         <v>43.579999999999991</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="37" t="s">
         <v>151</v>
       </c>
@@ -48851,7 +48902,7 @@
         <v>43.699999999999996</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="37" t="s">
         <v>151</v>
       </c>
@@ -48871,7 +48922,7 @@
         <v>43.599999999999994</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="37" t="s">
         <v>151</v>
       </c>
@@ -48891,7 +48942,7 @@
         <v>43.599999999999994</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="37" t="s">
         <v>151</v>
       </c>
@@ -48911,7 +48962,7 @@
         <v>43.59</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="37" t="s">
         <v>151</v>
       </c>
@@ -48931,7 +48982,7 @@
         <v>43.56</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="37" t="s">
         <v>164</v>
       </c>
@@ -48951,7 +49002,7 @@
         <v>44.31</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="37" t="s">
         <v>164</v>
       </c>
@@ -48971,7 +49022,7 @@
         <v>44.97999999999999</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="37" t="s">
         <v>164</v>
       </c>
@@ -48991,7 +49042,7 @@
         <v>45.329999999999991</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="37" t="s">
         <v>164</v>
       </c>
@@ -49011,7 +49062,7 @@
         <v>45.499999999999993</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="37" t="s">
         <v>164</v>
       </c>
@@ -49031,7 +49082,7 @@
         <v>45.57</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="37" t="s">
         <v>164</v>
       </c>
@@ -49051,7 +49102,7 @@
         <v>45.699999999999996</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="37" t="s">
         <v>164</v>
       </c>
@@ -49071,7 +49122,7 @@
         <v>45.87</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="37" t="s">
         <v>164</v>
       </c>
@@ -49091,7 +49142,7 @@
         <v>46.03</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="37" t="s">
         <v>164</v>
       </c>
@@ -49111,7 +49162,7 @@
         <v>46.189999999999991</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="37" t="s">
         <v>164</v>
       </c>
@@ -49131,7 +49182,7 @@
         <v>46.239999999999995</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="37" t="s">
         <v>164</v>
       </c>
@@ -49151,7 +49202,7 @@
         <v>46.31</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="37" t="s">
         <v>164</v>
       </c>
@@ -49171,7 +49222,7 @@
         <v>46.42</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="37" t="s">
         <v>177</v>
       </c>
@@ -49191,7 +49242,7 @@
         <v>46.699999999999996</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="37" t="s">
         <v>177</v>
       </c>
@@ -49211,7 +49262,7 @@
         <v>47.339999999999996</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="37" t="s">
         <v>177</v>
       </c>
@@ -49231,7 +49282,7 @@
         <v>47.839999999999996</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="37" t="s">
         <v>177</v>
       </c>
@@ -49251,7 +49302,7 @@
         <v>47.959999999999994</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="37" t="s">
         <v>177</v>
       </c>
@@ -49271,7 +49322,7 @@
         <v>47.97</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="37" t="s">
         <v>177</v>
       </c>
@@ -49291,7 +49342,7 @@
         <v>48.06</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="37" t="s">
         <v>177</v>
       </c>
@@ -49311,7 +49362,7 @@
         <v>48.159999999999989</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="37" t="s">
         <v>177</v>
       </c>
@@ -49331,7 +49382,7 @@
         <v>48.169999999999995</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="37" t="s">
         <v>177</v>
       </c>
@@ -49351,7 +49402,7 @@
         <v>48.259999999999991</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="37" t="s">
         <v>177</v>
       </c>
@@ -49371,7 +49422,7 @@
         <v>48.39</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="37" t="s">
         <v>177</v>
       </c>
@@ -49391,7 +49442,7 @@
         <v>48.39</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="37" t="s">
         <v>177</v>
       </c>
@@ -49411,7 +49462,7 @@
         <v>48.539999999999992</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="37" t="s">
         <v>190</v>
       </c>
@@ -49431,7 +49482,7 @@
         <v>49.429999999999993</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="37" t="s">
         <v>190</v>
       </c>
@@ -49451,7 +49502,7 @@
         <v>50.29</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="37" t="s">
         <v>190</v>
       </c>
@@ -49471,7 +49522,7 @@
         <v>50.639999999999993</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="37" t="s">
         <v>190</v>
       </c>
@@ -49491,7 +49542,7 @@
         <v>50.92</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="37" t="s">
         <v>190</v>
       </c>
@@ -49511,7 +49562,7 @@
         <v>51.04</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="37" t="s">
         <v>190</v>
       </c>
@@ -49531,7 +49582,7 @@
         <v>51.180000000000007</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="37" t="s">
         <v>190</v>
       </c>
@@ -49551,7 +49602,7 @@
         <v>51.31</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="37" t="s">
         <v>190</v>
       </c>
@@ -49571,7 +49622,7 @@
         <v>51.339999999999996</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="37" t="s">
         <v>190</v>
       </c>
@@ -49591,7 +49642,7 @@
         <v>51.239999999999995</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="37" t="s">
         <v>190</v>
       </c>
@@ -49611,7 +49662,7 @@
         <v>51.38</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="37" t="s">
         <v>190</v>
       </c>
@@ -49631,7 +49682,7 @@
         <v>51.6</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="37" t="s">
         <v>190</v>
       </c>
@@ -49651,7 +49702,7 @@
         <v>51.65</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="37" t="s">
         <v>203</v>
       </c>
@@ -49671,7 +49722,7 @@
         <v>51.889999999999993</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="37" t="s">
         <v>203</v>
       </c>
@@ -49691,7 +49742,7 @@
         <v>52.94</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="37" t="s">
         <v>203</v>
       </c>
@@ -49711,7 +49762,7 @@
         <v>54.109999999999992</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="37" t="s">
         <v>203</v>
       </c>
@@ -49731,7 +49782,7 @@
         <v>54.589999999999996</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="37" t="s">
         <v>203</v>
       </c>
@@ -49751,7 +49802,7 @@
         <v>54.58</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="37" t="s">
         <v>203</v>
       </c>
@@ -49771,7 +49822,7 @@
         <v>54.709999999999994</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="37" t="s">
         <v>203</v>
       </c>
@@ -49791,7 +49842,7 @@
         <v>54.84</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="37" t="s">
         <v>203</v>
       </c>
@@ -49811,7 +49862,7 @@
         <v>54.75</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="37" t="s">
         <v>203</v>
       </c>
@@ -49831,7 +49882,7 @@
         <v>54.829999999999991</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="37" t="s">
         <v>203</v>
       </c>
@@ -49851,7 +49902,7 @@
         <v>54.97</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="37" t="s">
         <v>203</v>
       </c>
@@ -49871,7 +49922,7 @@
         <v>55.469999999999985</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="37" t="s">
         <v>203</v>
       </c>
@@ -49891,7 +49942,7 @@
         <v>55.419999999999995</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="37" t="s">
         <v>216</v>
       </c>
@@ -49911,7 +49962,7 @@
         <v>55.81</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="37" t="s">
         <v>216</v>
       </c>
@@ -49931,7 +49982,7 @@
         <v>56.84</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="37" t="s">
         <v>216</v>
       </c>
@@ -49951,7 +50002,7 @@
         <v>57.629999999999995</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="37" t="s">
         <v>216</v>
       </c>
@@ -49971,7 +50022,7 @@
         <v>57.999999999999993</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="37" t="s">
         <v>216</v>
       </c>
@@ -49991,7 +50042,7 @@
         <v>58.239999999999995</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="37" t="s">
         <v>216</v>
       </c>
@@ -50011,7 +50062,7 @@
         <v>58.28</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="37" t="s">
         <v>216</v>
       </c>
@@ -50031,7 +50082,7 @@
         <v>58.69</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="37" t="s">
         <v>216</v>
       </c>
@@ -50051,7 +50102,7 @@
         <v>59.17</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="37" t="s">
         <v>216</v>
       </c>
@@ -50071,7 +50122,7 @@
         <v>59.249999999999993</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="37" t="s">
         <v>216</v>
       </c>
@@ -50091,7 +50142,7 @@
         <v>59.209999999999994</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="37" t="s">
         <v>216</v>
       </c>
@@ -50111,7 +50162,7 @@
         <v>59.36999999999999</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="37" t="s">
         <v>216</v>
       </c>
@@ -50131,7 +50182,7 @@
         <v>59.69</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="37" t="s">
         <v>229</v>
       </c>
@@ -50151,7 +50202,7 @@
         <v>60.289999999999985</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="37" t="s">
         <v>229</v>
       </c>
@@ -50171,7 +50222,7 @@
         <v>61.239999999999995</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="37" t="s">
         <v>229</v>
       </c>
@@ -50191,7 +50242,7 @@
         <v>61.919999999999995</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="37" t="s">
         <v>229</v>
       </c>
@@ -50211,7 +50262,7 @@
         <v>62.069999999999993</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="37" t="s">
         <v>229</v>
       </c>
@@ -50231,7 +50282,7 @@
         <v>62.129999999999995</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="37" t="s">
         <v>229</v>
       </c>
@@ -50251,7 +50302,7 @@
         <v>62.47999999999999</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="37" t="s">
         <v>229</v>
       </c>
@@ -50271,7 +50322,7 @@
         <v>62.82</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="37" t="s">
         <v>229</v>
       </c>
@@ -50291,7 +50342,7 @@
         <v>62.999999999999986</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="37" t="s">
         <v>229</v>
       </c>
@@ -50311,7 +50362,7 @@
         <v>63.61999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="37" t="s">
         <v>229</v>
       </c>
@@ -50331,7 +50382,7 @@
         <v>64.279999999999987</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="37" t="s">
         <v>229</v>
       </c>
@@ -50351,7 +50402,7 @@
         <v>64.34999999999998</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" s="37" t="s">
         <v>229</v>
       </c>
@@ -50371,7 +50422,7 @@
         <v>64.81</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" s="37" t="s">
         <v>242</v>
       </c>
@@ -50391,7 +50442,7 @@
         <v>65.19</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="37" t="s">
         <v>242</v>
       </c>
@@ -50411,7 +50462,7 @@
         <v>65.34999999999998</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="37" t="s">
         <v>242</v>
       </c>
@@ -50431,7 +50482,7 @@
         <v>65.789999999999992</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="37" t="s">
         <v>242</v>
       </c>
@@ -50451,7 +50502,7 @@
         <v>66.099999999999994</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="37" t="s">
         <v>242</v>
       </c>
@@ -50471,7 +50522,7 @@
         <v>66.399999999999991</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="37" t="s">
         <v>242</v>
       </c>
@@ -50491,7 +50542,7 @@
         <v>66.48</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="37" t="s">
         <v>242</v>
       </c>
@@ -50511,7 +50562,7 @@
         <v>66.88</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="37" t="s">
         <v>242</v>
       </c>
@@ -50531,7 +50582,7 @@
         <v>67.58</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="37" t="s">
         <v>242</v>
       </c>
@@ -50551,7 +50602,7 @@
         <v>67.789999999999992</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="37" t="s">
         <v>242</v>
       </c>
@@ -50571,7 +50622,7 @@
         <v>68.010000000000005</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" s="37" t="s">
         <v>242</v>
       </c>
@@ -50591,7 +50642,7 @@
         <v>68.20999999999998</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" s="37" t="s">
         <v>242</v>
       </c>
@@ -50611,7 +50662,7 @@
         <v>68.41</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" s="37" t="s">
         <v>255</v>
       </c>
@@ -50631,7 +50682,7 @@
         <v>68.97</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" s="37" t="s">
         <v>255</v>
       </c>
@@ -50651,7 +50702,7 @@
         <v>69.52</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" s="37" t="s">
         <v>255</v>
       </c>
@@ -50671,7 +50722,7 @@
         <v>69.789999999999992</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="37" t="s">
         <v>255</v>
       </c>
@@ -50691,7 +50742,7 @@
         <v>69.760000000000005</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" s="37" t="s">
         <v>255</v>
       </c>
@@ -50711,7 +50762,7 @@
         <v>70.22</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="37" t="s">
         <v>255</v>
       </c>
@@ -50731,7 +50782,7 @@
         <v>70.78</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" s="37" t="s">
         <v>255</v>
       </c>
@@ -50751,7 +50802,7 @@
         <v>71.040000000000006</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" s="37" t="s">
         <v>255</v>
       </c>
@@ -50771,7 +50822,7 @@
         <v>71.37</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="37" t="s">
         <v>255</v>
       </c>
@@ -50791,7 +50842,7 @@
         <v>71.45999999999998</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" s="37" t="s">
         <v>255</v>
       </c>
@@ -50811,7 +50862,7 @@
         <v>71.61</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" s="37" t="s">
         <v>255</v>
       </c>
@@ -50831,7 +50882,7 @@
         <v>71.569999999999993</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" s="37" t="s">
         <v>255</v>
       </c>
@@ -50851,7 +50902,7 @@
         <v>71.47999999999999</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" s="37" t="s">
         <v>268</v>
       </c>
@@ -50871,7 +50922,7 @@
         <v>71.650000000000006</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" s="37" t="s">
         <v>268</v>
       </c>
@@ -50891,7 +50942,7 @@
         <v>72.12</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" s="37" t="s">
         <v>268</v>
       </c>
@@ -50911,7 +50962,7 @@
         <v>72.489999999999981</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="37" t="s">
         <v>268</v>
       </c>
@@ -50931,7 +50982,7 @@
         <v>72.70999999999998</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="37" t="s">
         <v>268</v>
       </c>
@@ -50951,7 +51002,7 @@
         <v>72.769999999999982</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="37" t="s">
         <v>268</v>
       </c>
@@ -50971,7 +51022,7 @@
         <v>72.87</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="37" t="s">
         <v>268</v>
       </c>
@@ -50991,7 +51042,7 @@
         <v>73.009999999999991</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" s="37" t="s">
         <v>268</v>
       </c>
@@ -51011,7 +51062,7 @@
         <v>73.23</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" s="37" t="s">
         <v>268</v>
       </c>
@@ -51031,7 +51082,7 @@
         <v>73.469999999999985</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" s="37" t="s">
         <v>268</v>
       </c>
@@ -51051,7 +51102,7 @@
         <v>73.469999999999985</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="37" t="s">
         <v>268</v>
       </c>
@@ -51071,7 +51122,7 @@
         <v>73.650000000000006</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="37" t="s">
         <v>268</v>
       </c>
@@ -51091,7 +51142,7 @@
         <v>73.540000000000006</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" s="37" t="s">
         <v>12</v>
       </c>
@@ -51111,7 +51162,7 @@
         <v>73.7</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="37" t="s">
         <v>12</v>
       </c>
@@ -51131,7 +51182,7 @@
         <v>74.339999999999989</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="37" t="s">
         <v>12</v>
       </c>
@@ -51151,7 +51202,7 @@
         <v>74.5</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="37" t="s">
         <v>12</v>
       </c>
@@ -51171,7 +51222,7 @@
         <v>74.669999999999987</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" s="37" t="s">
         <v>12</v>
       </c>
@@ -51191,7 +51242,7 @@
         <v>74.92</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="37" t="s">
         <v>12</v>
       </c>
@@ -51211,7 +51262,7 @@
         <v>74.84999999999998</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" s="37" t="s">
         <v>12</v>
       </c>
@@ -51231,7 +51282,7 @@
         <v>74.72999999999999</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="37" t="s">
         <v>12</v>
       </c>
@@ -51251,7 +51302,7 @@
         <v>74.639999999999986</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" s="37" t="s">
         <v>12</v>
       </c>
@@ -51271,7 +51322,7 @@
         <v>74.819999999999979</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" s="37" t="s">
         <v>12</v>
       </c>
@@ -51291,7 +51342,7 @@
         <v>75.069999999999993</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" s="37" t="s">
         <v>12</v>
       </c>
@@ -51311,7 +51362,7 @@
         <v>75.249999999999986</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" s="37" t="s">
         <v>12</v>
       </c>
@@ -51331,7 +51382,7 @@
         <v>75.409999999999982</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" s="37" t="s">
         <v>13</v>
       </c>
@@ -51351,7 +51402,7 @@
         <v>75.499999999999986</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" s="37" t="s">
         <v>13</v>
       </c>
@@ -51371,7 +51422,7 @@
         <v>75.73</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" s="37" t="s">
         <v>13</v>
       </c>
@@ -51391,7 +51442,7 @@
         <v>75.859999999999985</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" s="37" t="s">
         <v>13</v>
       </c>
@@ -51411,7 +51462,7 @@
         <v>76.109999999999985</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" s="37" t="s">
         <v>13</v>
       </c>
@@ -51431,7 +51482,7 @@
         <v>76.709999999999994</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" s="37" t="s">
         <v>13</v>
       </c>
@@ -51451,7 +51502,7 @@
         <v>76.91</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" s="37" t="s">
         <v>13</v>
       </c>
@@ -51471,7 +51522,7 @@
         <v>76.999999999999986</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="37" t="s">
         <v>13</v>
       </c>
@@ -51491,7 +51542,7 @@
         <v>77.27</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" s="37" t="s">
         <v>13</v>
       </c>
@@ -51511,7 +51562,7 @@
         <v>77.84</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" s="37" t="s">
         <v>13</v>
       </c>
@@ -51531,7 +51582,7 @@
         <v>78.219999999999985</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" s="37" t="s">
         <v>13</v>
       </c>
@@ -51551,7 +51602,7 @@
         <v>79.149999999999991</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" s="37" t="s">
         <v>13</v>
       </c>
@@ -51571,7 +51622,7 @@
         <v>79.66</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" s="37" t="s">
         <v>14</v>
       </c>
@@ -51591,7 +51642,7 @@
         <v>79.650000000000006</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" s="37" t="s">
         <v>14</v>
       </c>
@@ -51611,7 +51662,7 @@
         <v>80.299999999999983</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" s="37" t="s">
         <v>14</v>
       </c>
@@ -51631,7 +51682,7 @@
         <v>81.12</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" s="37" t="s">
         <v>14</v>
       </c>
@@ -51651,7 +51702,7 @@
         <v>81.569999999999993</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" s="37" t="s">
         <v>14</v>
       </c>
@@ -51671,7 +51722,7 @@
         <v>81.749999999999986</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" s="37" t="s">
         <v>14</v>
       </c>
@@ -51691,7 +51742,7 @@
         <v>81.89</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" s="37" t="s">
         <v>14</v>
       </c>
@@ -51711,7 +51762,7 @@
         <v>82.02</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" s="37" t="s">
         <v>14</v>
       </c>
@@ -51731,7 +51782,7 @@
         <v>82.39</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" s="37" t="s">
         <v>14</v>
       </c>
@@ -51751,7 +51802,7 @@
         <v>82.829999999999984</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" s="37" t="s">
         <v>14</v>
       </c>
@@ -51771,7 +51822,7 @@
         <v>83.59</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" s="37" t="s">
         <v>14</v>
       </c>
@@ -51791,7 +51842,7 @@
         <v>84.179999999999993</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" s="37" t="s">
         <v>14</v>
       </c>
@@ -51811,7 +51862,7 @@
         <v>84.2</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" s="37" t="s">
         <v>15</v>
       </c>
@@ -51831,7 +51882,7 @@
         <v>85.759999999999991</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" s="37" t="s">
         <v>15</v>
       </c>
@@ -51851,7 +51902,7 @@
         <v>89.699999999999989</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" s="37" t="s">
         <v>15</v>
       </c>
@@ -51871,7 +51922,7 @@
         <v>93.269999999999982</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" s="37" t="s">
         <v>15</v>
       </c>
@@ -51891,7 +51942,7 @@
         <v>95.329999999999984</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" s="37" t="s">
         <v>15</v>
       </c>
@@ -51911,7 +51962,7 @@
         <v>95.999999999999986</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" s="37" t="s">
         <v>15</v>
       </c>
@@ -51931,7 +51982,7 @@
         <v>96.469999999999985</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212" s="37" t="s">
         <v>15</v>
       </c>
@@ -51951,7 +52002,7 @@
         <v>96.969999999999985</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" s="37" t="s">
         <v>15</v>
       </c>
@@ -51971,7 +52022,7 @@
         <v>97.249999999999986</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" s="37" t="s">
         <v>15</v>
       </c>
@@ -51991,7 +52042,7 @@
         <v>97.509999999999991</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215" s="37" t="s">
         <v>15</v>
       </c>
@@ -52011,7 +52062,7 @@
         <v>97.589999999999989</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A216" s="37" t="s">
         <v>15</v>
       </c>
@@ -52031,7 +52082,7 @@
         <v>97.669999999999987</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217" s="37" t="s">
         <v>15</v>
       </c>
@@ -52051,7 +52102,7 @@
         <v>97.91</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" s="37" t="s">
         <v>16</v>
       </c>
@@ -52071,7 +52122,7 @@
         <v>98.559999999999974</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219" s="37" t="s">
         <v>16</v>
       </c>
@@ -52091,7 +52142,7 @@
         <v>99.069999999999979</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220" s="37" t="s">
         <v>16</v>
       </c>
@@ -52111,7 +52162,7 @@
         <v>99.39</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" s="37" t="s">
         <v>16</v>
       </c>
@@ -52131,7 +52182,7 @@
         <v>99.399999999999991</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" s="37" t="s">
         <v>16</v>
       </c>
@@ -52151,7 +52202,7 @@
         <v>99.39</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" s="37" t="s">
         <v>16</v>
       </c>
@@ -52171,7 +52222,7 @@
         <v>99.659999999999982</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" s="37" t="s">
         <v>16</v>
       </c>
@@ -52191,7 +52242,7 @@
         <v>99.44</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A225" s="37" t="s">
         <v>16</v>
       </c>
@@ -52211,7 +52262,7 @@
         <v>99.169999999999987</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A226" s="37" t="s">
         <v>16</v>
       </c>
@@ -52231,7 +52282,7 @@
         <v>99.399999999999991</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A227" s="37" t="s">
         <v>16</v>
       </c>
@@ -52251,7 +52302,7 @@
         <v>99.36</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A228" s="37" t="s">
         <v>16</v>
       </c>
@@ -52271,7 +52322,7 @@
         <v>99.769999999999982</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A229" s="37" t="s">
         <v>16</v>
       </c>
@@ -52291,7 +52342,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A230" s="37" t="s">
         <v>17</v>
       </c>
@@ -52311,7 +52362,7 @@
         <v>99.72999999999999</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A231" s="37" t="s">
         <v>17</v>
       </c>
@@ -52331,7 +52382,7 @@
         <v>101.16999999999999</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A232" s="37" t="s">
         <v>17</v>
       </c>
@@ -52351,7 +52402,7 @@
         <v>106.03</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A233" s="37" t="s">
         <v>17</v>
       </c>
@@ -52371,7 +52422,7 @@
         <v>109.83000000000001</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A234" s="37" t="s">
         <v>17</v>
       </c>
@@ -52391,7 +52442,7 @@
         <v>110.7</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A235" s="37" t="s">
         <v>17</v>
       </c>
@@ -52411,7 +52462,7 @@
         <v>111.44999999999999</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A236" s="37" t="s">
         <v>17</v>
       </c>
@@ -52431,7 +52482,7 @@
         <v>111.55999999999999</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A237" s="37" t="s">
         <v>17</v>
       </c>
@@ -52451,7 +52502,7 @@
         <v>111.16999999999999</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A238" s="37" t="s">
         <v>17</v>
       </c>
@@ -52471,7 +52522,7 @@
         <v>110.46999999999998</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A239" s="37" t="s">
         <v>17</v>
       </c>
@@ -52491,7 +52542,7 @@
         <v>110.62999999999998</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A240" s="37" t="s">
         <v>17</v>
       </c>
@@ -52511,7 +52562,7 @@
         <v>110.74</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A241" s="37" t="s">
         <v>17</v>
       </c>
@@ -52531,7 +52582,7 @@
         <v>110.81999999999998</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A242" s="37" t="s">
         <v>18</v>
       </c>
@@ -52551,7 +52602,7 @@
         <v>110.72999999999999</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A243" s="37" t="s">
         <v>18</v>
       </c>
@@ -52571,7 +52622,7 @@
         <v>110.9</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244" s="37" t="s">
         <v>18</v>
       </c>
@@ -52591,7 +52642,7 @@
         <v>111.46999999999998</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" s="37" t="s">
         <v>18</v>
       </c>
@@ -52611,7 +52662,7 @@
         <v>112.07999999999998</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A246" s="37" t="s">
         <v>18</v>
       </c>
@@ -52631,7 +52682,7 @@
         <v>112.18999999999998</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A247" s="37" t="s">
         <v>18</v>
       </c>
@@ -52651,7 +52702,7 @@
         <v>112.06999999999998</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A248" s="37" t="s">
         <v>18</v>
       </c>
@@ -52671,7 +52722,7 @@
         <v>111.95999999999997</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A249" s="37" t="s">
         <v>18</v>
       </c>
@@ -52691,7 +52742,7 @@
         <v>111.89999999999998</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250" s="37" t="s">
         <v>18</v>
       </c>
@@ -52711,7 +52762,7 @@
         <v>112.07999999999998</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" s="37" t="s">
         <v>18</v>
       </c>
@@ -52731,7 +52782,7 @@
         <v>111.87999999999998</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A252" s="37" t="s">
         <v>18</v>
       </c>
@@ -52751,7 +52802,7 @@
         <v>111.32</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A253" s="37" t="s">
         <v>18</v>
       </c>
@@ -52771,7 +52822,7 @@
         <v>111.21999999999998</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254" s="37" t="s">
         <v>19</v>
       </c>
@@ -52791,7 +52842,7 @@
         <v>111.23</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255" s="37" t="s">
         <v>19</v>
       </c>
@@ -52811,7 +52862,7 @@
         <v>111.5</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256" s="37" t="s">
         <v>19</v>
       </c>
@@ -52831,7 +52882,7 @@
         <v>111.92</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257" s="37" t="s">
         <v>19</v>
       </c>
@@ -52851,7 +52902,7 @@
         <v>112.07999999999998</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A258" s="37" t="s">
         <v>19</v>
       </c>
@@ -52871,7 +52922,7 @@
         <v>112.53</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A259" s="37" t="s">
         <v>19</v>
       </c>
@@ -52891,7 +52942,7 @@
         <v>112.96</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A260" s="37" t="s">
         <v>19</v>
       </c>
@@ -52911,7 +52962,7 @@
         <v>112.99999999999999</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A261" s="37" t="s">
         <v>19</v>
       </c>
@@ -52931,7 +52982,7 @@
         <v>113.10999999999997</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A262" s="37" t="s">
         <v>19</v>
       </c>
@@ -52951,7 +53002,7 @@
         <v>113.19</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A263" s="37" t="s">
         <v>19</v>
       </c>
@@ -52971,7 +53022,7 @@
         <v>113.25</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A264" s="37" t="s">
         <v>19</v>
       </c>
@@ -52991,7 +53042,7 @@
         <v>113.22999999999999</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A265" s="37" t="s">
         <v>19</v>
       </c>
@@ -53011,7 +53062,7 @@
         <v>113.32999999999997</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A266" s="37" t="s">
         <v>20</v>
       </c>
@@ -53031,7 +53082,7 @@
         <v>113.41999999999999</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A267" s="37" t="s">
         <v>20</v>
       </c>
@@ -53051,7 +53102,7 @@
         <v>113.77</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A268" s="37" t="s">
         <v>20</v>
       </c>
@@ -53071,7 +53122,7 @@
         <v>114.90999999999998</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A269" s="37" t="s">
         <v>20</v>
       </c>
@@ -53091,7 +53142,7 @@
         <v>115.82999999999998</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A270" s="37" t="s">
         <v>20</v>
       </c>
@@ -53111,7 +53162,7 @@
         <v>116.31999999999998</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A271" s="37" t="s">
         <v>20</v>
       </c>
@@ -53131,7 +53182,7 @@
         <v>116.58999999999999</v>
       </c>
     </row>
-    <row r="272" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A272" s="37" t="s">
         <v>20</v>
       </c>
@@ -53151,7 +53202,7 @@
         <v>116.93</v>
       </c>
     </row>
-    <row r="273" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A273" s="37" t="s">
         <v>20</v>
       </c>
@@ -53171,7 +53222,7 @@
         <v>117.15</v>
       </c>
     </row>
-    <row r="274" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A274" s="37" t="s">
         <v>20</v>
       </c>
@@ -53191,7 +53242,7 @@
         <v>117.55</v>
       </c>
     </row>
-    <row r="275" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A275" s="37" t="s">
         <v>20</v>
       </c>
@@ -53211,7 +53262,7 @@
         <v>117.95</v>
       </c>
     </row>
-    <row r="276" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A276" s="37" t="s">
         <v>20</v>
       </c>
@@ -53231,7 +53282,7 @@
         <v>118.12</v>
       </c>
     </row>
-    <row r="277" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A277" s="37" t="s">
         <v>20</v>
       </c>
@@ -53251,7 +53302,7 @@
         <v>118.25</v>
       </c>
     </row>
-    <row r="278" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A278" s="37" t="s">
         <v>21</v>
       </c>
@@ -53271,7 +53322,7 @@
         <v>118.38</v>
       </c>
     </row>
-    <row r="279" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A279" s="37" t="s">
         <v>21</v>
       </c>
@@ -53291,7 +53342,7 @@
         <v>120.31</v>
       </c>
     </row>
-    <row r="280" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A280" s="37" t="s">
         <v>21</v>
       </c>
@@ -53311,7 +53362,7 @@
         <v>123.78</v>
       </c>
     </row>
-    <row r="281" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A281" s="37" t="s">
         <v>21</v>
       </c>
@@ -53331,7 +53382,7 @@
         <v>126.22</v>
       </c>
     </row>
-    <row r="282" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A282" s="37" t="s">
         <v>21</v>
       </c>
@@ -53351,7 +53402,7 @@
         <v>127.65</v>
       </c>
     </row>
-    <row r="283" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A283" s="37" t="s">
         <v>21</v>
       </c>
@@ -53371,7 +53422,7 @@
         <v>127.95</v>
       </c>
     </row>
-    <row r="284" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A284" s="37" t="s">
         <v>21</v>
       </c>
@@ -53391,7 +53442,7 @@
         <v>128.18</v>
       </c>
     </row>
-    <row r="285" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A285" s="37" t="s">
         <v>21</v>
       </c>
@@ -53411,7 +53462,7 @@
         <v>128.55000000000001</v>
       </c>
     </row>
-    <row r="286" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A286" s="37" t="s">
         <v>21</v>
       </c>
@@ -53431,7 +53482,7 @@
         <v>128.72999999999999</v>
       </c>
     </row>
-    <row r="287" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A287" s="37" t="s">
         <v>21</v>
       </c>
@@ -53451,7 +53502,7 @@
         <v>129.06</v>
       </c>
     </row>
-    <row r="288" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A288" s="37" t="s">
         <v>21</v>
       </c>
@@ -53471,7 +53522,7 @@
         <v>129.65</v>
       </c>
     </row>
-    <row r="289" spans="1:6" ht="15" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A289" s="37" t="s">
         <v>21</v>
       </c>
@@ -53503,14 +53554,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A953639D-114A-48EB-98DB-EE132607A951}">
   <dimension ref="A1:O13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -53533,7 +53584,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2013</v>
       </c>
@@ -53548,7 +53599,7 @@
         <v>9.8000000000000309E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2014</v>
       </c>
@@ -53556,7 +53607,7 @@
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -53566,7 +53617,7 @@
       </c>
       <c r="E4" s="6"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2016</v>
       </c>
@@ -53574,7 +53625,7 @@
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -53582,7 +53633,7 @@
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -53590,7 +53641,7 @@
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2019</v>
       </c>
@@ -53603,7 +53654,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2020</v>
       </c>
@@ -53616,7 +53667,7 @@
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -53629,7 +53680,7 @@
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -53642,12 +53693,12 @@
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2023</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B13" s="57" t="s">
         <v>407</v>
       </c>
@@ -53674,17 +53725,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="57ed4d19-7dfa-4218-b0c9-321a76363151">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f52a8275-2cbd-4186-978c-53e036657375" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010027EAE559E09D4A429EBD0F39DC21BBA6" ma:contentTypeVersion="16" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="c9719185c29a5bbeaf569b57ce7223ff">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="57ed4d19-7dfa-4218-b0c9-321a76363151" xmlns:ns3="f52a8275-2cbd-4186-978c-53e036657375" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6164b0d521ef8826ab87409b1a303be5" ns2:_="" ns3:_="">
     <xsd:import namespace="57ed4d19-7dfa-4218-b0c9-321a76363151"/>
@@ -53927,6 +53967,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="57ed4d19-7dfa-4218-b0c9-321a76363151">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f52a8275-2cbd-4186-978c-53e036657375" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -53937,17 +53988,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B018C194-A9E7-4F06-ABD3-76ED67C36641}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="57ed4d19-7dfa-4218-b0c9-321a76363151"/>
-    <ds:schemaRef ds:uri="f52a8275-2cbd-4186-978c-53e036657375"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DC54314F-D1AC-4123-9DE9-1A3CC599CBAF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -53966,6 +54006,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B018C194-A9E7-4F06-ABD3-76ED67C36641}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="57ed4d19-7dfa-4218-b0c9-321a76363151"/>
+    <ds:schemaRef ds:uri="f52a8275-2cbd-4186-978c-53e036657375"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{561C49FA-4DD9-4C75-A7B3-259135C5DB72}">
   <ds:schemaRefs>

</xml_diff>